<commit_message>
Model and tracker: remove explanatory italic notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/files/ironbend-buyer-tracker.xlsx
+++ b/public/files/ironbend-buyer-tracker.xlsx
@@ -199,7 +199,7 @@
     <t>VISUAL SUMMARY  —  LIVE CHARTS (LINKED TO BUYER TRACKER)</t>
   </si>
   <si>
-    <t>Chart source data (auto — mirrors the boxes above; do not edit)</t>
+    <t>Chart Data</t>
   </si>
   <si>
     <t>Active</t>
@@ -2587,7 +2587,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i/>
       <sz val="9"/>
       <color rgb="FF808080"/>
       <name val="Arial"/>
@@ -2640,7 +2639,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i/>
       <sz val="8"/>
       <color rgb="FFBF8F00"/>
       <name val="Arial"/>
@@ -2671,7 +2669,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i/>
       <sz val="7"/>
       <color rgb="FF808080"/>
       <name val="Arial"/>
@@ -2709,7 +2706,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i/>
       <sz val="8"/>
       <color rgb="FF808080"/>
       <name val="Arial"/>
@@ -2724,7 +2720,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i/>
       <sz val="7"/>
       <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
@@ -2785,7 +2780,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i/>
       <sz val="8"/>
       <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
@@ -2799,7 +2793,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i/>
       <sz val="9"/>
       <color rgb="FF2F5597"/>
       <name val="Arial"/>
@@ -5331,9 +5324,7 @@
     </row>
     <row r="36" spans="1:11" ht="25.5" customHeight="1">
       <c r="A36" s="16"/>
-      <c r="B36" s="83" t="s">
-        <v>823</v>
-      </c>
+      <c r="B36" s="83"/>
       <c r="C36" s="83"/>
       <c r="D36" s="83"/>
       <c r="E36" s="83"/>
@@ -5544,9 +5535,7 @@
       <c r="X1" s="14"/>
     </row>
     <row r="2" spans="1:24" ht="13.5" customHeight="1">
-      <c r="A2" s="86" t="s">
-        <v>808</v>
-      </c>
+      <c r="A2" s="86"/>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
       <c r="D2" s="86"/>
@@ -13950,9 +13939,7 @@
       <c r="I24" s="88"/>
     </row>
     <row r="26" spans="1:9" ht="39.75" customHeight="1">
-      <c r="A26" s="91" t="s">
-        <v>714</v>
-      </c>
+      <c r="A26" s="91"/>
       <c r="B26" s="91"/>
       <c r="C26" s="91"/>
       <c r="D26" s="91"/>
@@ -14007,9 +13994,7 @@
       <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" ht="13.5" customHeight="1">
-      <c r="A2" s="13" t="s">
-        <v>716</v>
-      </c>
+      <c r="A2" s="13"/>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>

</xml_diff>